<commit_message>
fix: revise chapter 4 per author review
- Broaden standardization definition (R08 note), add z(0.75) = 0.674 to
  memorized values (R40 note), introduce lepto-/meso-/platykurtic (R48)
- Clarify tails, independent mu/sigma, NORM.S.DIST vs NORM.DIST and density,
  sten/stanine rounding procedure; use "mez" for interval endpoints
- Show the Q-Q example in the principle section; add left-skewed and
  light-tailed simulations with verified quantile distortions
- Extend standard-score figure to z = -3..3, label band shares and
  cumulative shares in the sten/stanine figure
- Update workbook (two Sim_ sheets), checks, overviews and author docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_04.xlsx
+++ b/data/kapitola_04.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33B62199-8425-4B8B-890F-0EDC01EE7FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C144945-8A9B-4502-831F-D27AD408A4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{E165FF1A-5F0A-49E9-A088-3B78EC568C0A}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{4A0A6F10-B855-443F-A03E-A1F9BEA70190}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,8 @@
     <sheet name="Sim_sikme" sheetId="19" r:id="rId19"/>
     <sheet name="Sim_chvosty" sheetId="20" r:id="rId20"/>
     <sheet name="Sim_smes" sheetId="21" r:id="rId21"/>
+    <sheet name="Sim_sikme_vlevo" sheetId="22" r:id="rId22"/>
+    <sheet name="Sim_lehke" sheetId="23" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="135">
   <si>
     <t>Normální model</t>
   </si>
@@ -83,13 +85,13 @@
     <t>Přímý převod na podíl</t>
   </si>
   <si>
-    <t>Dolní hranice (body)</t>
-  </si>
-  <si>
-    <t>Horní hranice (body)</t>
-  </si>
-  <si>
-    <t>Podíl mezi hranicemi</t>
+    <t>Dolní mez (body)</t>
+  </si>
+  <si>
+    <t>Horní mez (body)</t>
+  </si>
+  <si>
+    <t>Podíl mezi mezemi</t>
   </si>
   <si>
     <t>Podíl vlevo</t>
@@ -110,12 +112,6 @@
     <t>Podíl v jednom chvostu</t>
   </si>
   <si>
-    <t>Dolní mez (body)</t>
-  </si>
-  <si>
-    <t>Horní mez (body)</t>
-  </si>
-  <si>
     <t>Autorský ilustrační model skóru pozornosti.</t>
   </si>
   <si>
@@ -444,6 +440,12 @@
   </si>
   <si>
     <t>Sim_smes</t>
+  </si>
+  <si>
+    <t>Sim_sikme_vlevo</t>
+  </si>
+  <si>
+    <t>Sim_lehke</t>
   </si>
   <si>
     <t>A1:D25</t>
@@ -787,7 +789,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-95A6-40DD-A3E5-F863981A32F3}"/>
+              <c16:uniqueId val="{00000008-9256-44C1-94FC-FB2158D72C35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -901,7 +903,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-95A6-40DD-A3E5-F863981A32F3}"/>
+              <c16:uniqueId val="{00000009-9256-44C1-94FC-FB2158D72C35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -913,11 +915,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="883778752"/>
-        <c:axId val="883780672"/>
+        <c:axId val="1164856047"/>
+        <c:axId val="1164867567"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="883778752"/>
+        <c:axId val="1164856047"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2"/>
@@ -947,13 +949,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="883780672"/>
+        <c:crossAx val="1164867567"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="883780672"/>
+        <c:axId val="1164867567"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -981,7 +983,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="883778752"/>
+        <c:crossAx val="1164856047"/>
         <c:crossesAt val="-2"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1180,7 +1182,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-5D1E-41BF-AB08-D3562C30A25F}"/>
+              <c16:uniqueId val="{00000008-8AE5-4A1E-AC68-9000AE458192}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1294,7 +1296,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-5D1E-41BF-AB08-D3562C30A25F}"/>
+              <c16:uniqueId val="{00000009-8AE5-4A1E-AC68-9000AE458192}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1306,11 +1308,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1695869903"/>
-        <c:axId val="1695872783"/>
+        <c:axId val="1164868047"/>
+        <c:axId val="1164864207"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1695869903"/>
+        <c:axId val="1164868047"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1340,13 +1342,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1695872783"/>
+        <c:crossAx val="1164864207"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1695872783"/>
+        <c:axId val="1164864207"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1376,7 +1378,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1695869903"/>
+        <c:crossAx val="1164868047"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
@@ -1439,7 +1441,7 @@
         <xdr:cNvPr id="2" name="Graf 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{040D4174-3722-268F-56DF-4B97B205973C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2A79358-AF4E-7A75-A44F-6445F2BF10F6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1475,7 +1477,7 @@
         <xdr:cNvPr id="3" name="Graf 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BB7C2C4-5A7E-C207-B493-230EBB0329A5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C7D836E-DF92-0645-F46E-14BB2019E792}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1812,8 +1814,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEC759E7-29C3-4B04-A857-C3D0C6A96419}">
-  <dimension ref="A1:C30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC0D22CF-D47E-4A75-B463-15DA91FAD1B8}">
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="25.625" customWidth="1"/>
@@ -1822,7 +1824,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1834,277 +1836,299 @@
     </row>
     <row r="3" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
     </row>
     <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B4" s="19"/>
       <c r="C4" s="19"/>
     </row>
     <row r="5" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
     </row>
     <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
     </row>
     <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>54</v>
+        <v>128</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
     </row>
     <row r="30" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2119,7 +2143,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C82B95-3B33-4010-8314-72191CB408AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B748F50A-6420-4E90-9FA9-A0D7CD1F0D94}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2129,10 +2153,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2140,7 +2164,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2154,7 +2178,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2182,7 +2206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A58480-5BC6-4F86-AAA8-40A08A10A12C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E910E5-A7EA-46E2-B9D9-C1736470A5C6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2193,13 +2217,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2210,7 +2234,7 @@
         <v>80</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2224,13 +2248,13 @@
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B4" s="14">
         <v>0.08</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2244,7 +2268,7 @@
     </row>
     <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" s="14">
         <v>25</v>
@@ -2264,7 +2288,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6AB753-2C1C-4C8E-840D-9B25C76BB77D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0B69289-AA34-4DAC-9BEE-8F3B8A5803DD}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2275,13 +2299,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2292,7 +2316,7 @@
         <v>50</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2306,18 +2330,18 @@
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B4" s="14">
         <v>45</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B5" s="14">
         <v>65</v>
@@ -2326,7 +2350,7 @@
     </row>
     <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" s="14">
         <v>20</v>
@@ -2335,7 +2359,7 @@
     </row>
     <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B7" s="14">
         <v>8</v>
@@ -2352,7 +2376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3936583F-D594-4C23-9660-AB8EC155A6DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78D8E3D3-546F-4A6C-AD33-66F8A2F80212}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2363,13 +2387,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2380,7 +2404,7 @@
         <v>50</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2400,12 +2424,12 @@
         <v>0.2</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="14">
         <v>0.1</v>
@@ -2434,7 +2458,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2626B2D-E3CA-43E0-8B6C-3963C1CC9F31}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79986BEA-76C8-4AD1-B44A-B6C7819420F2}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2445,13 +2469,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2462,7 +2486,7 @@
         <v>50</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2476,18 +2500,18 @@
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="14">
         <v>50</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B5" s="14">
         <v>1</v>
@@ -2510,7 +2534,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABB95700-F352-4E62-B217-0B56CF2143E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FDAE8B7-77C0-4C72-B2EA-90A234D545B7}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2520,10 +2544,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2531,7 +2555,7 @@
         <v>38</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2545,7 +2569,7 @@
         <v>60</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2570,7 +2594,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40ACB1AE-ACBB-4347-AFF0-62E135F55DE1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A303A4A-A3B5-4525-A43F-660AC44E0F1F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2580,10 +2604,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2591,7 +2615,7 @@
         <v>1.2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2605,7 +2629,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2627,7 +2651,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95530D35-B61C-4308-B4F2-3742B7ACEB47}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92A2BDE6-7B4C-449C-AAAE-555802B61CF4}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2637,10 +2661,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2648,7 +2672,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2662,7 +2686,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2723,7 +2747,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36DE2AB6-FADC-4B0C-BC8E-1CEA3ED8EA67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E828F21-B68F-4E38-A94E-ECC0917A572A}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2733,10 +2757,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2744,7 +2768,7 @@
         <v>48.85602655957382</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2758,7 +2782,7 @@
         <v>29.327651524791108</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3759,7 +3783,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2261A7-86A8-49E7-8BCB-CEB28EA0B313}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E76D6B6-F167-402B-8BDE-5F02A7D14F80}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3769,10 +3793,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3780,7 +3804,7 @@
         <v>66.073597304495223</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3794,7 +3818,7 @@
         <v>80.020527650875579</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4795,7 +4819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C8580E3-BC35-4CE3-B51B-75E91D498FF4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F894E161-84B4-4807-93E3-0CEA1F45BF2D}">
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4827,7 +4851,7 @@
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -4841,7 +4865,7 @@
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -4863,7 +4887,7 @@
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -4891,7 +4915,7 @@
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4906,7 +4930,7 @@
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -4929,7 +4953,7 @@
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -4943,7 +4967,7 @@
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -4978,7 +5002,7 @@
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -5085,7 +5109,7 @@
     </row>
     <row r="24" spans="1:6" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B24" s="9">
         <f>_xlfn.NORM.INV(B23,B2,B3)</f>
@@ -5098,7 +5122,7 @@
     </row>
     <row r="25" spans="1:6" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B25" s="9">
         <f>_xlfn.NORM.INV(1-B23,B2,B3)</f>
@@ -5147,7 +5171,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C33B4A1C-4578-44C5-BDC8-8F47C4E52632}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C2E6DD1-5EE5-4142-AEE5-8E3011462CAA}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5157,10 +5181,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5168,7 +5192,7 @@
         <v>44.583323970004095</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5182,7 +5206,7 @@
         <v>22.049299769270561</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6183,7 +6207,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01D3D00-2798-491C-BDE7-C7C8787D5FA4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130DFEC5-EC78-4A0A-846D-285700F57BB0}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6193,10 +6217,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6204,7 +6228,7 @@
         <v>36.276933564652332</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6218,7 +6242,7 @@
         <v>35.639479476123725</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7207,6 +7231,2078 @@
     <row r="201" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="18">
         <v>62.217355862155749</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F3CFAA-E4F1-4676-97C7-96704803B99F}">
+  <dimension ref="A1:C201"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
+        <v>68.15406359732151</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18">
+        <v>65.903256717137992</v>
+      </c>
+      <c r="C3" s="16"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
+        <v>63.971926025114954</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
+        <v>63.684091111645103</v>
+      </c>
+      <c r="C5" s="16"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
+        <v>44.085506481447453</v>
+      </c>
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
+        <v>66.256279135122895</v>
+      </c>
+      <c r="C7" s="16"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
+        <v>69.003366821229676</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
+        <v>30.66381408252645</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
+        <v>64.901006795548994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
+        <v>69.439091901294887</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
+        <v>57.748960871669517</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18">
+        <v>65.837693950161338</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18">
+        <v>59.622667422938221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18">
+        <v>51.881279685443403</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18">
+        <v>63.323133820667863</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
+        <v>69.770360249094665</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18">
+        <v>63.672768254764378</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18">
+        <v>21.836418325739373</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="18">
+        <v>67.852026061154902</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18">
+        <v>69.40068556429209</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="18">
+        <v>68.862554035149515</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="18">
+        <v>61.330015398199969</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
+        <v>59.749066923233741</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="18">
+        <v>67.303809864563547</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="18">
+        <v>37.665798516761775</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="18">
+        <v>61.422756836238385</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="18">
+        <v>66.229441935704969</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="18">
+        <v>65.365416743070568</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="18">
+        <v>69.163908791731359</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="18">
+        <v>66.183201628737152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="18">
+        <v>48.499367964782948</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="18">
+        <v>69.989033644087613</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="18">
+        <v>63.89130306430161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="18">
+        <v>63.073906661011279</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="18">
+        <v>61.292501417452378</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="18">
+        <v>63.190186279825866</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="18">
+        <v>65.417461488395929</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="18">
+        <v>64.997382666915655</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="18">
+        <v>69.372790437191725</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="18">
+        <v>67.213252182118595</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="18">
+        <v>68.628837061114609</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="18">
+        <v>64.152404759079218</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="18">
+        <v>69.186743353493512</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="18">
+        <v>50.647774171924354</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="18">
+        <v>62.881567078131319</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="18">
+        <v>64.536593542434275</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="18">
+        <v>66.237899428233504</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="18">
+        <v>69.82309999410063</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="18">
+        <v>66.381855397485197</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="18">
+        <v>53.309334070330621</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="18">
+        <v>44.723450673141713</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="18">
+        <v>68.318493459373713</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="18">
+        <v>27.141006703215112</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="18">
+        <v>59.166635116982334</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="18">
+        <v>49.21822575936293</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="18">
+        <v>67.251667319796979</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="18">
+        <v>64.051090343855321</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="18">
+        <v>69.163206345401704</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="18">
+        <v>60.187724819826961</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="18">
+        <v>67.126636286266148</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="18">
+        <v>68.19448544178158</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="18">
+        <v>61.934845401394249</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="18">
+        <v>67.325844308122299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="18">
+        <v>48.592788783231015</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="18">
+        <v>68.80921034142375</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="18">
+        <v>53.927314915603162</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="18">
+        <v>67.184346038848162</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="18">
+        <v>64.984008702449501</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="18">
+        <v>68.681420953944325</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="18">
+        <v>57.162500620308393</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="18">
+        <v>28.56183136092065</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="18">
+        <v>64.845928973518312</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="18">
+        <v>33.860786308682705</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="18">
+        <v>64.824970536865294</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="18">
+        <v>69.035267727449536</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="18">
+        <v>69.860888523980975</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="18">
+        <v>60.814164150926352</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="18">
+        <v>62.222131687605568</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="18">
+        <v>54.138825876698739</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="18">
+        <v>51.774967835193635</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="18">
+        <v>60.725120949047685</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="18">
+        <v>60.442665107968331</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="18">
+        <v>43.09331620238089</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="18">
+        <v>61.08277672943759</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="18">
+        <v>68.599343481473625</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="18">
+        <v>69.957813219505113</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="18">
+        <v>67.37631868892575</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="18">
+        <v>63.806246984750032</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="18">
+        <v>65.007871212437749</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="18">
+        <v>59.400562998327487</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="18">
+        <v>60.050475104200721</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="18">
+        <v>61.36010745424295</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="18">
+        <v>63.697921088896692</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="18">
+        <v>61.835123121765385</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="18">
+        <v>66.162578742951155</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="18">
+        <v>63.177781314589083</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="18">
+        <v>67.223013770733857</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="18">
+        <v>26.952396220120814</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="18">
+        <v>61.409417828965069</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="18">
+        <v>63.939713072031736</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="18">
+        <v>69.711294073748903</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="18">
+        <v>50.358935502266647</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="18">
+        <v>63.675325699150562</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="18">
+        <v>65.740929935127497</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="18">
+        <v>60.318842409598709</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="18">
+        <v>63.164688120596111</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="18">
+        <v>69.720857515164695</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="18">
+        <v>68.172278606654459</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="18">
+        <v>55.127329473292583</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="18">
+        <v>66.689402391541037</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="18">
+        <v>59.711335748854154</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="18">
+        <v>69.785951757803559</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="18">
+        <v>68.368981926155584</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="18">
+        <v>57.907977281558388</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="18">
+        <v>69.502522514836613</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="18">
+        <v>67.168812085874379</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="18">
+        <v>65.109582911289735</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="18">
+        <v>60.784521822038627</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="18">
+        <v>63.621471753819804</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="18">
+        <v>44.529263657846691</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="18">
+        <v>61.603337453598513</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="18">
+        <v>62.634366974654675</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="18">
+        <v>65.707171722315252</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="18">
+        <v>59.883957868862026</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="18">
+        <v>47.089721250855106</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="18">
+        <v>64.135908745229244</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="18">
+        <v>64.498678483068943</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="18">
+        <v>64.617446279153228</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="18">
+        <v>64.589405474252999</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="18">
+        <v>64.495418764636554</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="18">
+        <v>65.157488510012627</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="18">
+        <v>39.731272088181491</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="18">
+        <v>55.10317601470755</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="18">
+        <v>69.921586601994932</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="18">
+        <v>65.377256562933326</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="18">
+        <v>52.137102764940025</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="18">
+        <v>66.093358634971082</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="18">
+        <v>65.959082841873169</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="18">
+        <v>49.534032569175714</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="18">
+        <v>68.630873506959176</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="18">
+        <v>64.701181864365935</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="18">
+        <v>66.375338637310961</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="18">
+        <v>37.786630244743343</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="18">
+        <v>63.989662388339639</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="18">
+        <v>51.505820603018762</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="18">
+        <v>66.653778995387256</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="18">
+        <v>69.501903397031128</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="18">
+        <v>54.403790757900232</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="18">
+        <v>54.168964737003797</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="18">
+        <v>54.282969572490209</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="18">
+        <v>67.931337301499255</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="18">
+        <v>62.979649250558928</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="18">
+        <v>66.799648582177852</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="18">
+        <v>59.304515130608635</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="18">
+        <v>67.52361168153584</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="18">
+        <v>59.393040184351683</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="18">
+        <v>63.56746275909245</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="18">
+        <v>55.512787704458688</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="18">
+        <v>67.87473007074253</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="18">
+        <v>66.220361185260117</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="18">
+        <v>38.301261739623058</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="18">
+        <v>37.205278949629779</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="18">
+        <v>63.673041500151157</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="18">
+        <v>53.906791336942867</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="18">
+        <v>67.224547651763274</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="18">
+        <v>58.577946769493693</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="18">
+        <v>66.639596014283597</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="18">
+        <v>10.622601284424263</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="18">
+        <v>53.714845344670209</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="18">
+        <v>64.480729224160314</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="18">
+        <v>69.245125320740044</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="18">
+        <v>67.549383253416266</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="18">
+        <v>69.457086031325161</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="18">
+        <v>61.83220518794942</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="18">
+        <v>55.901519344023789</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="18">
+        <v>68.253622539460679</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="18">
+        <v>57.730194107118123</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="18">
+        <v>60.565905193624573</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="18">
+        <v>36.330436544310565</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="18">
+        <v>54.371732604598755</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="18">
+        <v>68.076506294310093</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="18">
+        <v>66.814738283865154</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="18">
+        <v>64.854898252524436</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="18">
+        <v>52.315707635974647</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="18">
+        <v>54.665355068540329</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="18">
+        <v>53.966292260536029</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="18">
+        <v>67.771987211088117</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="18">
+        <v>19.593071681097499</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="18">
+        <v>43.101171237745518</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="18">
+        <v>64.850421641021967</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="18">
+        <v>68.547247480636074</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="18">
+        <v>61.988776791668542</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="18">
+        <v>66.080443824692964</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="18">
+        <v>54.670921345182563</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="18">
+        <v>69.752130196429789</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="18">
+        <v>66.856773183866252</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="18">
+        <v>67.858769148588181</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="18">
+        <v>63.998540183529258</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="18">
+        <v>52.715792879839704</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="18">
+        <v>47.550380483448464</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F6BEEB4-665F-447C-961F-1F125E5D68DF}">
+  <dimension ref="A1:C201"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
+        <v>54.159601153805852</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18">
+        <v>66.380661819130182</v>
+      </c>
+      <c r="C3" s="16"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
+        <v>36.291775908321142</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
+        <v>50.686198230832815</v>
+      </c>
+      <c r="C5" s="16"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
+        <v>31.592826182022691</v>
+      </c>
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
+        <v>45.855253227055073</v>
+      </c>
+      <c r="C7" s="16"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
+        <v>30.320517616346478</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
+        <v>52.302951691672206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
+        <v>49.434026712551713</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
+        <v>43.199387555941939</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
+        <v>56.002839189022779</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18">
+        <v>63.57905781827867</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18">
+        <v>32.869030348956585</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18">
+        <v>58.837524456903338</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18">
+        <v>69.796532960608602</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
+        <v>47.778660459443927</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18">
+        <v>63.368809698149562</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18">
+        <v>68.03225489333272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="18">
+        <v>43.620424745604403</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18">
+        <v>59.179010717198253</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="18">
+        <v>54.713209187611938</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="18">
+        <v>39.906998192891479</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
+        <v>54.700477113947272</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="18">
+        <v>65.905556287616491</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="18">
+        <v>48.372254511341453</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="18">
+        <v>69.898928459733725</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="18">
+        <v>63.934656400233507</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="18">
+        <v>50.923178065568209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="18">
+        <v>46.912962635979056</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="18">
+        <v>63.923185840249062</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="18">
+        <v>40.89056265540421</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="18">
+        <v>41.869257381185889</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="18">
+        <v>48.810077300295234</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="18">
+        <v>55.641898140311241</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="18">
+        <v>35.514342486858368</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="18">
+        <v>33.811726784333587</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="18">
+        <v>47.603143313899629</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="18">
+        <v>48.058695737272501</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="18">
+        <v>46.699465122073889</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="18">
+        <v>55.661057541146874</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="18">
+        <v>65.828026421368122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="18">
+        <v>34.533796273171902</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="18">
+        <v>49.820895986631513</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="18">
+        <v>68.34688963368535</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="18">
+        <v>59.393338020890951</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="18">
+        <v>42.243235912173986</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="18">
+        <v>55.272279866039753</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="18">
+        <v>35.142013486474752</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="18">
+        <v>43.110614437609911</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="18">
+        <v>69.392444984987378</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="18">
+        <v>40.75867997482419</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="18">
+        <v>48.73500338755548</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="18">
+        <v>31.786803537979718</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="18">
+        <v>31.982082910835743</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="18">
+        <v>55.842280834913254</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="18">
+        <v>66.566613717004657</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="18">
+        <v>59.079321585595608</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="18">
+        <v>53.112175399437547</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="18">
+        <v>66.850007614120841</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="18">
+        <v>39.644232336431742</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="18">
+        <v>67.799554318189621</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="18">
+        <v>59.231163468211889</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="18">
+        <v>65.581199442967772</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="18">
+        <v>35.482415361329913</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="18">
+        <v>55.319436984136701</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="18">
+        <v>33.917870698496699</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="18">
+        <v>67.946593435481191</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="18">
+        <v>46.660039061680429</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="18">
+        <v>62.638314943760633</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="18">
+        <v>55.942162619903677</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="18">
+        <v>67.160349432379007</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="18">
+        <v>69.526862446218729</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="18">
+        <v>53.961099330335855</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="18">
+        <v>52.42811388336122</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="18">
+        <v>50.728246290236712</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="18">
+        <v>41.554477345198393</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="18">
+        <v>48.927850946784019</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="18">
+        <v>37.299285233020782</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="18">
+        <v>62.793126543983817</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="18">
+        <v>61.664043515920639</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="18">
+        <v>40.086802085861571</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="18">
+        <v>37.580863414332271</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="18">
+        <v>39.40100310370326</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="18">
+        <v>64.929334465414286</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="18">
+        <v>38.812923701480031</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="18">
+        <v>56.085501546040177</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="18">
+        <v>49.970622388646007</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="18">
+        <v>39.551843293011189</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="18">
+        <v>44.322796929627657</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="18">
+        <v>69.830646272748709</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="18">
+        <v>33.525597183033824</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="18">
+        <v>54.766030581668019</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="18">
+        <v>56.523997485637665</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="18">
+        <v>63.554204320535064</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="18">
+        <v>53.303320398554206</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="18">
+        <v>55.987999374046922</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="18">
+        <v>69.871886996552348</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="18">
+        <v>57.877961648628109</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="18">
+        <v>48.032662989571691</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="18">
+        <v>47.323811231181026</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="18">
+        <v>51.103584431111813</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="18">
+        <v>67.10775782354176</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="18">
+        <v>61.860852492973208</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="18">
+        <v>42.269951719790697</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="18">
+        <v>56.52883805334568</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="18">
+        <v>59.640783695504069</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="18">
+        <v>57.985356627032161</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="18">
+        <v>52.775864265859127</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="18">
+        <v>69.65032079257071</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="18">
+        <v>38.445673892274499</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="18">
+        <v>51.816422147676349</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="18">
+        <v>52.66826044768095</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="18">
+        <v>46.604007706046104</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="18">
+        <v>51.137546300888062</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="18">
+        <v>38.558493498712778</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="18">
+        <v>49.867883129045367</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="18">
+        <v>49.223454156890512</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="18">
+        <v>34.964152798056602</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="18">
+        <v>56.913818707689643</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="18">
+        <v>46.752912066876888</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="18">
+        <v>59.240476069971919</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="18">
+        <v>52.775810984894633</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="18">
+        <v>68.899649083614349</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="18">
+        <v>52.95214562676847</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="18">
+        <v>59.829586436972022</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="18">
+        <v>45.553642669692643</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="18">
+        <v>56.208467623218894</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="18">
+        <v>69.552129628136754</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="18">
+        <v>48.518926370888948</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="18">
+        <v>38.388260584324598</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="18">
+        <v>48.723424477502704</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="18">
+        <v>48.934789504855871</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="18">
+        <v>47.384428307414055</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="18">
+        <v>50.525541407987475</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="18">
+        <v>46.097106197848909</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="18">
+        <v>53.338918257504702</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="18">
+        <v>40.904699936509132</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="18">
+        <v>68.991130376234651</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="18">
+        <v>39.466299256309867</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="18">
+        <v>65.018547754734755</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="18">
+        <v>37.706687552854419</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="18">
+        <v>68.892200365662575</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="18">
+        <v>33.690879996865988</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="18">
+        <v>44.44531537592411</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="18">
+        <v>52.778187086805701</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="18">
+        <v>35.68511039018631</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="18">
+        <v>34.605477172881365</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="18">
+        <v>62.452744031324983</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="18">
+        <v>39.397408347576857</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="18">
+        <v>53.602568507194519</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="18">
+        <v>41.857693074271083</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="18">
+        <v>42.494654655456543</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="18">
+        <v>63.70848510414362</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="18">
+        <v>66.304153650999069</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="18">
+        <v>33.204325661063194</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="18">
+        <v>52.994925091043115</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="18">
+        <v>35.711140288040042</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="18">
+        <v>62.1308125089854</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="18">
+        <v>67.610325580462813</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="18">
+        <v>49.242674261331558</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="18">
+        <v>44.160215891897678</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="18">
+        <v>30.822160728275776</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="18">
+        <v>50.132974106818438</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="18">
+        <v>68.218390541151166</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="18">
+        <v>47.14512700214982</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="18">
+        <v>60.579321729019277</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="18">
+        <v>45.781482821330428</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="18">
+        <v>55.657301694154739</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="18">
+        <v>35.594209851697087</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="18">
+        <v>41.1560018081218</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="18">
+        <v>35.156222796067595</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="18">
+        <v>64.276959728449583</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="18">
+        <v>36.610254775732749</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="18">
+        <v>61.994597408920527</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="18">
+        <v>46.422534650191665</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="18">
+        <v>64.49917258694768</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="18">
+        <v>64.428684301674366</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="18">
+        <v>69.050594232976437</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="18">
+        <v>33.706649420782924</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="18">
+        <v>44.193472033366561</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="18">
+        <v>31.614128211513162</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="18">
+        <v>44.478811724111438</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="18">
+        <v>32.498178854584694</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="18">
+        <v>35.630365908145905</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="18">
+        <v>41.808858495205641</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="18">
+        <v>57.326766448095441</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="18">
+        <v>36.020947201177478</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="18">
+        <v>47.873855493962765</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="18">
+        <v>56.80857784114778</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="18">
+        <v>55.882668988779187</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="18">
+        <v>54.589489782229066</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="18">
+        <v>69.549052882939577</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="18">
+        <v>52.304007112979889</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="18">
+        <v>43.794741509482265</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="18">
+        <v>46.870538676157594</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="18">
+        <v>36.246237857267261</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="18">
+        <v>60.91596039943397</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="18">
+        <v>37.118570785969496</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="18">
+        <v>41.947133084759123</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="18">
+        <v>48.764944039285183</v>
       </c>
     </row>
   </sheetData>
@@ -7219,7 +9315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C955F2F1-43C9-4F71-B669-1BE51AD809F7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D389AD84-D528-4727-A4E4-AEB12F8E073E}">
   <dimension ref="A1:N44"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7234,22 +9330,22 @@
   <sheetData>
     <row r="1" spans="1:14" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -7284,7 +9380,7 @@
         <v>4.769730764606428E-2</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H2" s="12">
         <f>COUNT(B2:B13)</f>
@@ -7321,7 +9417,7 @@
         <v>0.11068209655016407</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H3" s="6">
         <f>AVERAGE(B2:B13)</f>
@@ -7358,7 +9454,7 @@
         <v>0.18689726251601743</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H4" s="6">
         <f>_xlfn.STDEV.S(B2:B13)</f>
@@ -7693,7 +9789,7 @@
     </row>
     <row r="16" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -7727,7 +9823,7 @@
     </row>
     <row r="18" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -7745,7 +9841,7 @@
     </row>
     <row r="19" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -7779,7 +9875,7 @@
     </row>
     <row r="21" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -7797,7 +9893,7 @@
     </row>
     <row r="22" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -7831,7 +9927,7 @@
     </row>
     <row r="24" spans="1:14" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -8174,7 +10270,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B127E1C0-C15F-44EB-AF34-589FAF6EC930}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE8459E6-98D4-4C0A-80A7-110A95963DFA}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8184,10 +10280,10 @@
   <sheetData>
     <row r="1" spans="1:6" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>2</v>
@@ -8196,12 +10292,12 @@
         <v>3</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="14">
         <v>60</v>
@@ -8213,12 +10309,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" s="14">
         <v>42</v>
@@ -8233,7 +10329,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -8255,7 +10351,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E736E3B-C501-4318-B90E-1A395ED65A30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2ACB657-8380-46F3-B107-5CCBEAE85396}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8265,10 +10361,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8276,7 +10372,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8290,7 +10386,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8318,7 +10414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C1634D-F83A-45C5-8EE7-D99343FB5988}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D876A9B-38B5-4E28-B3A6-873A143D0C9D}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8328,10 +10424,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8339,7 +10435,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8353,7 +10449,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8429,7 +10525,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BC518FD-1DE2-43D8-BFAF-75317D2A1417}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8048A5D2-78A7-4CE2-82C6-4041A76EC6C4}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8439,7 +10535,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>2</v>
@@ -8448,12 +10544,12 @@
         <v>3</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" s="14">
         <v>50</v>
@@ -8462,12 +10558,12 @@
         <v>10</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" s="14">
         <v>65</v>
@@ -8479,7 +10575,7 @@
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" s="14">
         <v>50</v>
@@ -8488,7 +10584,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -8510,7 +10606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FACE664-974F-4E86-90E6-D73B6AB7E193}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A962CF91-33A4-48CB-AF77-2D81DB22305B}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8520,21 +10616,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" s="14">
         <v>0</v>
@@ -8543,12 +10639,12 @@
         <v>1</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="14">
         <v>50</v>
@@ -8560,7 +10656,7 @@
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B4" s="14">
         <v>100</v>
@@ -8569,12 +10665,12 @@
         <v>15</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B5" s="14">
         <v>10</v>
@@ -8600,7 +10696,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E104B4FA-42D2-468E-8CCA-A100AF1CEB7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB6F9EE-22CD-46F6-93A0-BD6076AF6F2C}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8610,10 +10706,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>2</v>
@@ -8622,15 +10718,15 @@
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="14">
         <v>62</v>
@@ -8645,12 +10741,12 @@
         <v>-0.75</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" s="14">
         <v>62</v>
@@ -8666,7 +10762,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G4" s="17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Nahradit simulaci těžších chvostů výběrem s oběma těžkými konci
Původní výběr z 50 + 8·t (3 st. v.) ukazoval těžký chvost jen nahoře,
takže rozdíl data − model u 1. percentilu byl +0,4. Nový výběr z téhož
modelu (seed 20263319, tvořen až po ostatních simulacích) dává −6,9
u 1. a +7,9 u 99. percentilu, SKEW 0,01 a KURT 3,23. Upraven text,
alternativní popis, obě tabulky, věta o nestálosti excesu, kontroly
a sešit kapitoly 4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_04.xlsx
+++ b/data/kapitola_04.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C144945-8A9B-4502-831F-D27AD408A4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E73D967A-EDA1-4BF7-975B-53CCA69D6358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{4A0A6F10-B855-443F-A03E-A1F9BEA70190}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{B6B0A2F2-3418-4F22-89B5-CB9A06F1899A}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -789,7 +789,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-9256-44C1-94FC-FB2158D72C35}"/>
+              <c16:uniqueId val="{00000008-73EC-4EB7-A9D0-6C792A6A4238}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -903,7 +903,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-9256-44C1-94FC-FB2158D72C35}"/>
+              <c16:uniqueId val="{00000009-73EC-4EB7-A9D0-6C792A6A4238}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -915,11 +915,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1164856047"/>
-        <c:axId val="1164867567"/>
+        <c:axId val="606791583"/>
+        <c:axId val="606794463"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1164856047"/>
+        <c:axId val="606791583"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2"/>
@@ -949,13 +949,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1164867567"/>
+        <c:crossAx val="606794463"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1164867567"/>
+        <c:axId val="606794463"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -983,7 +983,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1164856047"/>
+        <c:crossAx val="606791583"/>
         <c:crossesAt val="-2"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1182,7 +1182,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-8AE5-4A1E-AC68-9000AE458192}"/>
+              <c16:uniqueId val="{00000008-0901-4282-AF84-53BD840002AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1296,7 +1296,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-8AE5-4A1E-AC68-9000AE458192}"/>
+              <c16:uniqueId val="{00000009-0901-4282-AF84-53BD840002AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1308,11 +1308,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1164868047"/>
-        <c:axId val="1164864207"/>
+        <c:axId val="606793503"/>
+        <c:axId val="606793983"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1164868047"/>
+        <c:axId val="606793503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1342,13 +1342,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1164864207"/>
+        <c:crossAx val="606793983"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1164864207"/>
+        <c:axId val="606793983"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1378,7 +1378,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
-        <c:crossAx val="1164868047"/>
+        <c:crossAx val="606793503"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.2"/>
@@ -1441,7 +1441,7 @@
         <xdr:cNvPr id="2" name="Graf 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2A79358-AF4E-7A75-A44F-6445F2BF10F6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E2FDD63-8578-7C7F-1EB9-641ED2D5A4D2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1477,7 +1477,7 @@
         <xdr:cNvPr id="3" name="Graf 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C7D836E-DF92-0645-F46E-14BB2019E792}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D5E2609-07D4-C8B0-8A48-56B7C91DFD4F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1814,7 +1814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC0D22CF-D47E-4A75-B463-15DA91FAD1B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25DDAA9D-FB87-484A-88E5-6AC619A7A1D8}">
   <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2143,7 +2143,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B748F50A-6420-4E90-9FA9-A0D7CD1F0D94}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B131DD71-16B5-4390-8B5C-318B0ADDBC07}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2206,7 +2206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E910E5-A7EA-46E2-B9D9-C1736470A5C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0237FC15-1280-4C86-BD23-1A262506D3E6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2288,7 +2288,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0B69289-AA34-4DAC-9BEE-8F3B8A5803DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A237558D-8A06-4817-99FD-2DDEC5E069EB}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2376,7 +2376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78D8E3D3-546F-4A6C-AD33-66F8A2F80212}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A1EEAC6-4518-45F1-8093-6C7A613F995E}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2458,7 +2458,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79986BEA-76C8-4AD1-B44A-B6C7819420F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE83EE95-E4D4-4092-9724-138565C8A087}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2534,7 +2534,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FDAE8B7-77C0-4C72-B2EA-90A234D545B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4532CD1B-F72D-4279-868D-8C3E85345C36}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2594,7 +2594,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A303A4A-A3B5-4525-A43F-660AC44E0F1F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB40D5EE-21B1-4D56-975B-804127A88850}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2651,7 +2651,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92A2BDE6-7B4C-449C-AAAE-555802B61CF4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03B14A65-0707-4542-BD9B-842C3CFC3BA8}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2747,7 +2747,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E828F21-B68F-4E38-A94E-ECC0917A572A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38EFCC64-6DEB-45C5-8E66-8FB88E67B0E0}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3783,7 +3783,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E76D6B6-F167-402B-8BDE-5F02A7D14F80}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B233DD26-5920-45CC-B28A-7625C6DA842A}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4819,7 +4819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F894E161-84B4-4807-93E3-0CEA1F45BF2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AA6035D-42F3-4081-B8C8-9BB9412D17E7}">
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5171,7 +5171,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C2E6DD1-5EE5-4142-AEE5-8E3011462CAA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FC6CA6-78EE-4020-83E6-90E14D4471C6}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5189,7 +5189,7 @@
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18">
-        <v>44.583323970004095</v>
+        <v>39.724727431511013</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>87</v>
@@ -5197,13 +5197,13 @@
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18">
-        <v>51.334447207766225</v>
+        <v>58.118776458561115</v>
       </c>
       <c r="C3" s="16"/>
     </row>
     <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18">
-        <v>22.049299769270561</v>
+        <v>51.549693565343112</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>88</v>
@@ -5211,990 +5211,990 @@
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18">
-        <v>67.12353898825269</v>
+        <v>54.168762503873189</v>
       </c>
       <c r="C5" s="16"/>
     </row>
     <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18">
-        <v>51.43348741741498</v>
+        <v>0.26450928128574702</v>
       </c>
       <c r="C6" s="16"/>
     </row>
     <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18">
-        <v>51.851061941192299</v>
+        <v>59.156280870021689</v>
       </c>
       <c r="C7" s="16"/>
     </row>
     <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18">
-        <v>61.899850011110217</v>
+        <v>51.00607829577649</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="18">
-        <v>45.089113454926675</v>
+        <v>58.368700636682519</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="18">
-        <v>58.022351957847448</v>
+        <v>53.672015724455157</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="18">
-        <v>27.918169643776512</v>
+        <v>50.891779514678191</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18">
-        <v>48.252400632490939</v>
+        <v>60.928077357477186</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="18">
-        <v>50.504048652608617</v>
+        <v>47.042420653698166</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18">
-        <v>46.940464063830234</v>
+        <v>60.370250101681357</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="18">
-        <v>32.477745204184998</v>
+        <v>54.789008326850976</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="18">
-        <v>47.776046232762582</v>
+        <v>53.75865911948803</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="18">
-        <v>52.364536146374576</v>
+        <v>59.222732716971443</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18">
-        <v>45.500856174103568</v>
+        <v>39.402243702258858</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="18">
-        <v>55.052096044162909</v>
+        <v>57.430363110897098</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="18">
-        <v>50.685613161086344</v>
+        <v>65.891015846816899</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="18">
-        <v>49.66952996775624</v>
+        <v>54.895824931083922</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18">
-        <v>104.0837872400076</v>
+        <v>54.1735664256802</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="18">
-        <v>48.138533562033437</v>
+        <v>42.715099022893277</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18">
-        <v>51.306818862784155</v>
+        <v>38.971480257404153</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18">
-        <v>50.20944889961028</v>
+        <v>44.268552042379582</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18">
-        <v>75.063939489551288</v>
+        <v>70.731069508894421</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="18">
-        <v>45.850919890213376</v>
+        <v>46.243143093170325</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="18">
-        <v>61.182874319803965</v>
+        <v>50.741456252539415</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="18">
-        <v>53.242645886564432</v>
+        <v>49.405084948705856</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="18">
-        <v>48.457622052033251</v>
+        <v>56.774428583154823</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="18">
-        <v>50.141780231489143</v>
+        <v>62.201435154424708</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="18">
-        <v>54.727203415741691</v>
+        <v>44.070829161996144</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="18">
-        <v>41.170085502511725</v>
+        <v>35.606389537296621</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="18">
-        <v>45.643499747389342</v>
+        <v>51.0817992094141</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="18">
-        <v>49.679103878592088</v>
+        <v>49.382484349741766</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="18">
-        <v>48.057261654852617</v>
+        <v>42.857879046631588</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="18">
-        <v>69.936980427049335</v>
+        <v>21.690969435868485</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18">
-        <v>49.69352250939118</v>
+        <v>45.798966644404146</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="18">
-        <v>68.62388039969656</v>
+        <v>48.934234645944727</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18">
-        <v>49.630861611768701</v>
+        <v>42.29757252431574</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="18">
-        <v>46.252110620339266</v>
+        <v>42.888432410652641</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="18">
-        <v>33.849920369473907</v>
+        <v>46.867880265574279</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="18">
-        <v>61.040272273906567</v>
+        <v>66.981012888387795</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="18">
-        <v>51.026349773822112</v>
+        <v>47.341479881702519</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="18">
-        <v>25.437813575006871</v>
+        <v>44.112392451074463</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="18">
-        <v>42.412842605243902</v>
+        <v>52.258088138642179</v>
       </c>
     </row>
     <row r="47" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="18">
-        <v>62.686303636400751</v>
+        <v>48.126382538297968</v>
       </c>
     </row>
     <row r="48" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="18">
-        <v>42.704975764121997</v>
+        <v>60.326213967587165</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="18">
-        <v>49.587829692225341</v>
+        <v>48.317790891858081</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="18">
-        <v>40.78205054740252</v>
+        <v>48.098361102434595</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="18">
-        <v>41.946539670316461</v>
+        <v>56.532791274604683</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="18">
-        <v>45.353919743322727</v>
+        <v>56.205372818910021</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="18">
-        <v>51.583911931211553</v>
+        <v>59.278661814366671</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="18">
-        <v>43.714457679757274</v>
+        <v>31.975622365288288</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="18">
-        <v>52.37259939470421</v>
+        <v>49.965090683132843</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="18">
-        <v>36.057837306818563</v>
+        <v>41.850920470666857</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="18">
-        <v>52.312866521311008</v>
+        <v>55.843622327535812</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="18">
-        <v>50.898708249164237</v>
+        <v>62.144257254596909</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="18">
-        <v>41.696665737883528</v>
+        <v>67.919104259787233</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="18">
-        <v>44.350601057959913</v>
+        <v>56.328545186684565</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="18">
-        <v>58.236466252153789</v>
+        <v>57.86354034888604</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="18">
-        <v>19.574030505252157</v>
+        <v>30.82231053339391</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="18">
-        <v>56.080188977948879</v>
+        <v>51.565234809090015</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="18">
-        <v>30.68074555636943</v>
+        <v>44.487758520778883</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="18">
-        <v>-12.204560354287352</v>
+        <v>52.097375011673627</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="18">
-        <v>45.220203620598937</v>
+        <v>43.094426157035976</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="18">
-        <v>17.633038518680848</v>
+        <v>42.403509176801457</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="18">
-        <v>52.558418096840398</v>
+        <v>50.78434181264182</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="18">
-        <v>53.918768547743881</v>
+        <v>58.422128835990357</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="18">
-        <v>56.972852118665365</v>
+        <v>51.846581487407626</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="18">
-        <v>58.026408528720026</v>
+        <v>51.001032356714063</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="18">
-        <v>42.542720247102906</v>
+        <v>98.625584203476706</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="18">
-        <v>48.323793455863751</v>
+        <v>50.223893813690545</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="18">
-        <v>50.092658671687573</v>
+        <v>27.181022851138508</v>
       </c>
     </row>
     <row r="75" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="18">
-        <v>45.229895119984732</v>
+        <v>61.374386747861536</v>
       </c>
     </row>
     <row r="76" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="18">
-        <v>52.728573385504006</v>
+        <v>55.046851001158039</v>
       </c>
     </row>
     <row r="77" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="18">
-        <v>71.899363117058016</v>
+        <v>53.319267573452812</v>
       </c>
     </row>
     <row r="78" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="18">
-        <v>44.513348927234212</v>
+        <v>64.121480066010079</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="18">
-        <v>63.77864435299476</v>
+        <v>47.990705362420563</v>
       </c>
     </row>
     <row r="80" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="18">
-        <v>46.436575656511899</v>
+        <v>60.40581371236064</v>
       </c>
     </row>
     <row r="81" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="18">
-        <v>34.887998227138411</v>
+        <v>62.495748118710729</v>
       </c>
     </row>
     <row r="82" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="18">
-        <v>58.462021678261699</v>
+        <v>53.351244138838112</v>
       </c>
     </row>
     <row r="83" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="18">
-        <v>88.463061624052457</v>
+        <v>82.14232343527209</v>
       </c>
     </row>
     <row r="84" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="18">
-        <v>67.934703645557789</v>
+        <v>50.582145829769068</v>
       </c>
     </row>
     <row r="85" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="18">
-        <v>42.4628425000082</v>
+        <v>42.392442026821755</v>
       </c>
     </row>
     <row r="86" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="18">
-        <v>61.204939847809861</v>
+        <v>52.232240301001326</v>
       </c>
     </row>
     <row r="87" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="18">
-        <v>30.712805609794103</v>
+        <v>45.09197018517721</v>
       </c>
     </row>
     <row r="88" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="18">
-        <v>51.861494525023879</v>
+        <v>54.948427753635393</v>
       </c>
     </row>
     <row r="89" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="18">
-        <v>54.918184385449301</v>
+        <v>32.246457508143337</v>
       </c>
     </row>
     <row r="90" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="18">
-        <v>32.623603626472288</v>
+        <v>55.981956745346146</v>
       </c>
     </row>
     <row r="91" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="18">
-        <v>45.728197050296096</v>
+        <v>42.737246373952154</v>
       </c>
     </row>
     <row r="92" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="18">
-        <v>43.597926883139415</v>
+        <v>38.93412277284262</v>
       </c>
     </row>
     <row r="93" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="18">
-        <v>23.030243265509871</v>
+        <v>46.595969605800896</v>
       </c>
     </row>
     <row r="94" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="18">
-        <v>56.656211338615392</v>
+        <v>35.488426913050532</v>
       </c>
     </row>
     <row r="95" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="18">
-        <v>58.795607188661208</v>
+        <v>50.584418788767863</v>
       </c>
     </row>
     <row r="96" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="18">
-        <v>45.169194495007787</v>
+        <v>60.34497695853851</v>
       </c>
     </row>
     <row r="97" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="18">
-        <v>58.697729354499721</v>
+        <v>57.396151120543223</v>
       </c>
     </row>
     <row r="98" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="18">
-        <v>36.002693637123954</v>
+        <v>70.475388241866398</v>
       </c>
     </row>
     <row r="99" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="18">
-        <v>48.499856032151719</v>
+        <v>53.91521312271513</v>
       </c>
     </row>
     <row r="100" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="18">
-        <v>55.574792339894898</v>
+        <v>48.174698978153863</v>
       </c>
     </row>
     <row r="101" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="18">
-        <v>46.620051006744809</v>
+        <v>38.949618607218184</v>
       </c>
     </row>
     <row r="102" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="18">
-        <v>35.192832980731971</v>
+        <v>46.389970981785247</v>
       </c>
     </row>
     <row r="103" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="18">
-        <v>45.186132660524521</v>
+        <v>54.290097759645406</v>
       </c>
     </row>
     <row r="104" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="18">
-        <v>41.440002205863252</v>
+        <v>52.471151283741023</v>
       </c>
     </row>
     <row r="105" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="18">
-        <v>56.867720158468678</v>
+        <v>45.442168206456557</v>
       </c>
     </row>
     <row r="106" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="18">
-        <v>53.295696930395053</v>
+        <v>35.499611058454988</v>
       </c>
     </row>
     <row r="107" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="18">
-        <v>64.889311035448912</v>
+        <v>46.495934367505633</v>
       </c>
     </row>
     <row r="108" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="18">
-        <v>54.26200612782938</v>
+        <v>52.704200478698787</v>
       </c>
     </row>
     <row r="109" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="18">
-        <v>52.544742047961151</v>
+        <v>44.419121975138992</v>
       </c>
     </row>
     <row r="110" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="18">
-        <v>40.523359873000345</v>
+        <v>61.149565185138883</v>
       </c>
     </row>
     <row r="111" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="18">
-        <v>46.446031997827333</v>
+        <v>51.046601593847974</v>
       </c>
     </row>
     <row r="112" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="18">
-        <v>51.779561027162579</v>
+        <v>48.492554319077684</v>
       </c>
     </row>
     <row r="113" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="18">
-        <v>49.014194362670722</v>
+        <v>51.421176174767488</v>
       </c>
     </row>
     <row r="114" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="18">
-        <v>61.819034752771493</v>
+        <v>63.835830736229738</v>
       </c>
     </row>
     <row r="115" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="18">
-        <v>29.985690829060811</v>
+        <v>49.125957357671297</v>
       </c>
     </row>
     <row r="116" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="18">
-        <v>53.876783794405526</v>
+        <v>39.766572080096871</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="18">
-        <v>61.539812338110224</v>
+        <v>36.18100292771112</v>
       </c>
     </row>
     <row r="118" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="18">
-        <v>43.974827192966821</v>
+        <v>46.340085968608527</v>
       </c>
     </row>
     <row r="119" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="18">
-        <v>45.551346114953439</v>
+        <v>58.571023212204665</v>
       </c>
     </row>
     <row r="120" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="18">
-        <v>50.084261318972246</v>
+        <v>56.158306536071883</v>
       </c>
     </row>
     <row r="121" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="18">
-        <v>62.01638668237868</v>
+        <v>32.705329596195241</v>
       </c>
     </row>
     <row r="122" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="18">
-        <v>56.175165413494142</v>
+        <v>46.330914380935489</v>
       </c>
     </row>
     <row r="123" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="18">
-        <v>47.456388751873405</v>
+        <v>55.358282433825607</v>
       </c>
     </row>
     <row r="124" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="18">
-        <v>23.038518892969723</v>
+        <v>35.030361414130681</v>
       </c>
     </row>
     <row r="125" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="18">
-        <v>51.998571819711955</v>
+        <v>50.289757718576865</v>
       </c>
     </row>
     <row r="126" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="18">
-        <v>44.601782349880828</v>
+        <v>59.053231030160973</v>
       </c>
     </row>
     <row r="127" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="18">
-        <v>62.587679284555179</v>
+        <v>43.621179876209631</v>
       </c>
     </row>
     <row r="128" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="18">
-        <v>47.981402959431179</v>
+        <v>55.381254103458886</v>
       </c>
     </row>
     <row r="129" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="18">
-        <v>57.746497474145698</v>
+        <v>54.273169688545877</v>
       </c>
     </row>
     <row r="130" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="18">
-        <v>39.268318019440855</v>
+        <v>54.434743771249067</v>
       </c>
     </row>
     <row r="131" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="18">
-        <v>40.593793682408517</v>
+        <v>42.422121465148308</v>
       </c>
     </row>
     <row r="132" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="18">
-        <v>68.981146636466704</v>
+        <v>56.2579563366982</v>
       </c>
     </row>
     <row r="133" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="18">
-        <v>52.193130853285872</v>
+        <v>52.736555807487591</v>
       </c>
     </row>
     <row r="134" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="18">
-        <v>33.76091170487512</v>
+        <v>57.402843295453799</v>
       </c>
     </row>
     <row r="135" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="18">
-        <v>50.171022483272182</v>
+        <v>47.395345262911022</v>
       </c>
     </row>
     <row r="136" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="18">
-        <v>60.620977113570738</v>
+        <v>55.028160532842065</v>
       </c>
     </row>
     <row r="137" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="18">
-        <v>39.784466650531179</v>
+        <v>51.172716178356914</v>
       </c>
     </row>
     <row r="138" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="18">
-        <v>63.595008502574217</v>
+        <v>48.374305284300064</v>
       </c>
     </row>
     <row r="139" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="18">
-        <v>50.529974380471813</v>
+        <v>15.108578494940213</v>
       </c>
     </row>
     <row r="140" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="18">
-        <v>44.190483929113618</v>
+        <v>71.120551635300288</v>
       </c>
     </row>
     <row r="141" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="18">
-        <v>53.542574514794453</v>
+        <v>69.910912378502431</v>
       </c>
     </row>
     <row r="142" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="18">
-        <v>39.477142117733074</v>
+        <v>50.143477787399455</v>
       </c>
     </row>
     <row r="143" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="18">
-        <v>43.732251991134852</v>
+        <v>57.087882553740172</v>
       </c>
     </row>
     <row r="144" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="18">
-        <v>41.959239458331346</v>
+        <v>30.37035360126303</v>
       </c>
     </row>
     <row r="145" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="18">
-        <v>38.792495139376115</v>
+        <v>43.287788272562587</v>
       </c>
     </row>
     <row r="146" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="18">
-        <v>45.854655573468918</v>
+        <v>43.714821159148705</v>
       </c>
     </row>
     <row r="147" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="18">
-        <v>60.354771536885288</v>
+        <v>55.22878609637408</v>
       </c>
     </row>
     <row r="148" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="18">
-        <v>62.219049231687123</v>
+        <v>16.744147548002623</v>
       </c>
     </row>
     <row r="149" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="18">
-        <v>45.52130275469495</v>
+        <v>45.623284594797433</v>
       </c>
     </row>
     <row r="150" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="18">
-        <v>49.924428774898615</v>
+        <v>44.418434899096489</v>
       </c>
     </row>
     <row r="151" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="18">
-        <v>37.764960053846963</v>
+        <v>80.906599676794229</v>
       </c>
     </row>
     <row r="152" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="18">
-        <v>51.658304855015182</v>
+        <v>48.851658693260283</v>
       </c>
     </row>
     <row r="153" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="18">
-        <v>29.707599198619079</v>
+        <v>50.255395651187406</v>
       </c>
     </row>
     <row r="154" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="18">
-        <v>46.231772923103257</v>
+        <v>48.366714535745814</v>
       </c>
     </row>
     <row r="155" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="18">
-        <v>55.298751839191588</v>
+        <v>38.138813119198225</v>
       </c>
     </row>
     <row r="156" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="18">
-        <v>41.922572445910873</v>
+        <v>62.114514106185744</v>
       </c>
     </row>
     <row r="157" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="18">
-        <v>48.262933858575977</v>
+        <v>89.044123304201307</v>
       </c>
     </row>
     <row r="158" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="18">
-        <v>44.476607929252594</v>
+        <v>46.230586871601425</v>
       </c>
     </row>
     <row r="159" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="18">
-        <v>48.533536089568322</v>
+        <v>50.297842099809216</v>
       </c>
     </row>
     <row r="160" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="18">
-        <v>50.891699221834102</v>
+        <v>54.532855937459317</v>
       </c>
     </row>
     <row r="161" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="18">
-        <v>55.942113835665133</v>
+        <v>87.757894474667111</v>
       </c>
     </row>
     <row r="162" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="18">
-        <v>46.056943456482507</v>
+        <v>54.466946468348141</v>
       </c>
     </row>
     <row r="163" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="18">
-        <v>58.216244888538114</v>
+        <v>50.471710169218099</v>
       </c>
     </row>
     <row r="164" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="18">
-        <v>52.217003100011731</v>
+        <v>62.42450312593202</v>
       </c>
     </row>
     <row r="165" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="18">
-        <v>48.210090208151811</v>
+        <v>47.861203939628588</v>
       </c>
     </row>
     <row r="166" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="18">
-        <v>62.0879827797365</v>
+        <v>51.513529406448818</v>
       </c>
     </row>
     <row r="167" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="18">
-        <v>64.228945367396022</v>
+        <v>76.547904892048948</v>
       </c>
     </row>
     <row r="168" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="18">
-        <v>20.131492243533419</v>
+        <v>53.242337114454543</v>
       </c>
     </row>
     <row r="169" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="18">
-        <v>110.64886999472245</v>
+        <v>48.247108662185646</v>
       </c>
     </row>
     <row r="170" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="18">
-        <v>32.941935085315933</v>
+        <v>57.160241955209123</v>
       </c>
     </row>
     <row r="171" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="18">
-        <v>38.163113947951629</v>
+        <v>67.311397552087669</v>
       </c>
     </row>
     <row r="172" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="18">
-        <v>28.014152026886876</v>
+        <v>45.750161515257368</v>
       </c>
     </row>
     <row r="173" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="18">
-        <v>37.31657769048735</v>
+        <v>25.695928137197193</v>
       </c>
     </row>
     <row r="174" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="18">
-        <v>62.196798206891565</v>
+        <v>34.168154301390146</v>
       </c>
     </row>
     <row r="175" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="18">
-        <v>71.437812193563587</v>
+        <v>50.758333896554582</v>
       </c>
     </row>
     <row r="176" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="18">
-        <v>60.833312973349301</v>
+        <v>36.42948761760335</v>
       </c>
     </row>
     <row r="177" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="18">
-        <v>47.624045845330549</v>
+        <v>34.495583143570343</v>
       </c>
     </row>
     <row r="178" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="18">
-        <v>47.969146974682602</v>
+        <v>46.070327372243071</v>
       </c>
     </row>
     <row r="179" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="18">
-        <v>41.411513183912675</v>
+        <v>47.321982102905089</v>
       </c>
     </row>
     <row r="180" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="18">
-        <v>40.775685771027305</v>
+        <v>65.168113679426</v>
       </c>
     </row>
     <row r="181" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="18">
-        <v>37.87482306899652</v>
+        <v>51.802903328288394</v>
       </c>
     </row>
     <row r="182" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="18">
-        <v>36.109009913511997</v>
+        <v>56.361311949642122</v>
       </c>
     </row>
     <row r="183" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="18">
-        <v>58.135307145492682</v>
+        <v>53.754812274581838</v>
       </c>
     </row>
     <row r="184" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="18">
-        <v>66.807164265069304</v>
+        <v>59.744493536762221</v>
       </c>
     </row>
     <row r="185" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="18">
-        <v>53.720121887290681</v>
+        <v>36.109468986345533</v>
       </c>
     </row>
     <row r="186" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="18">
-        <v>62.774840258291775</v>
+        <v>56.362964271399221</v>
       </c>
     </row>
     <row r="187" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="18">
-        <v>47.137994499823385</v>
+        <v>86.332687137693071</v>
       </c>
     </row>
     <row r="188" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="18">
-        <v>42.151912174740652</v>
+        <v>12.534328646608904</v>
       </c>
     </row>
     <row r="189" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="18">
-        <v>51.059677931739131</v>
+        <v>74.933317492812549</v>
       </c>
     </row>
     <row r="190" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="18">
-        <v>28.741581848902054</v>
+        <v>51.501287057655638</v>
       </c>
     </row>
     <row r="191" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="18">
-        <v>41.54036883231511</v>
+        <v>49.65016464913402</v>
       </c>
     </row>
     <row r="192" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="18">
-        <v>40.373172130813913</v>
+        <v>46.959105184612248</v>
       </c>
     </row>
     <row r="193" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="18">
-        <v>55.702822738870395</v>
+        <v>46.440390595706795</v>
       </c>
     </row>
     <row r="194" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="18">
-        <v>11.42434803408441</v>
+        <v>43.157416314777265</v>
       </c>
     </row>
     <row r="195" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="18">
-        <v>49.053571153044992</v>
+        <v>48.391180980109894</v>
       </c>
     </row>
     <row r="196" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="18">
-        <v>45.577680998383187</v>
+        <v>60.513406900320845</v>
       </c>
     </row>
     <row r="197" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="18">
-        <v>39.826789789901085</v>
+        <v>50.661008835384578</v>
       </c>
     </row>
     <row r="198" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="18">
-        <v>38.979676161116856</v>
+        <v>58.638692831012222</v>
       </c>
     </row>
     <row r="199" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="18">
-        <v>51.981276736960531</v>
+        <v>49.336674268847567</v>
       </c>
     </row>
     <row r="200" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="18">
-        <v>20.98298801463104</v>
+        <v>59.870246431122155</v>
       </c>
     </row>
     <row r="201" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="18">
-        <v>46.144000858098984</v>
+        <v>43.729801569967776</v>
       </c>
     </row>
   </sheetData>
@@ -6207,7 +6207,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130DFEC5-EC78-4A0A-846D-285700F57BB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA11DB-10CC-431D-AF32-89C62AABE066}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7243,7 +7243,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F3CFAA-E4F1-4676-97C7-96704803B99F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0FA0375-7537-41FB-BB68-5CF00F11F2D9}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8279,7 +8279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F6BEEB4-665F-447C-961F-1F125E5D68DF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{744FAFBB-E54B-49A5-9796-E58532FA182E}">
   <dimension ref="A1:C201"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -9315,7 +9315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D389AD84-D528-4727-A4E4-AEB12F8E073E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855D364F-ECB0-4D99-BA0E-60C3CE1D0027}">
   <dimension ref="A1:N44"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10270,7 +10270,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE8459E6-98D4-4C0A-80A7-110A95963DFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38288AB1-2B93-4D6A-97DB-856F390FA7B1}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10351,7 +10351,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2ACB657-8380-46F3-B107-5CCBEAE85396}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94D52721-F7B2-42F4-9737-2CCE66C8880C}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10414,7 +10414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D876A9B-38B5-4E28-B3A6-873A143D0C9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DAB06F5-8CA7-483A-B872-4714FF557BEA}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10525,7 +10525,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8048A5D2-78A7-4CE2-82C6-4041A76EC6C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F50F684-24C8-4D82-BCC6-55373D5B3B2D}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10606,7 +10606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A962CF91-33A4-48CB-AF77-2D81DB22305B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC99F7B8-73EC-4D44-9E0F-7FBF4670DFF8}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10696,7 +10696,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB6F9EE-22CD-46F6-93A0-BD6076AF6F2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1159BFD8-C8B7-46EE-A92D-F304D6761ABA}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>